<commit_message>
Logiciel de Assurance Automobile avec API ASAC. Modification du parmétrage de flotte avec l'option de modificatio complête des données de chaque véhicule
</commit_message>
<xml_diff>
--- a/modele_flotte_import.xlsx
+++ b/modele_flotte_import.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Véhicules" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Instructions" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,13 +26,23 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -46,8 +57,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,63 +427,142 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:V6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="15" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="20" customWidth="1" min="14" max="14"/>
+    <col width="15" customWidth="1" min="15" max="15"/>
+    <col width="25" customWidth="1" min="16" max="16"/>
+    <col width="9" customWidth="1" min="17" max="17"/>
+    <col width="24" customWidth="1" min="18" max="18"/>
+    <col width="13" customWidth="1" min="19" max="19"/>
+    <col width="17" customWidth="1" min="20" max="20"/>
+    <col width="22" customWidth="1" min="21" max="21"/>
+    <col width="19" customWidth="1" min="22" max="22"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>immatriculation</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>chassis</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>marque</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>modele</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>categorie</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>annee</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>energie</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>puissance</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>places</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>valeur_neuf</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>valeur_venale</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>categorie</t>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>type_vehicule</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>zone_tarifaire</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>proprietaire</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>telephone</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>ville</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>adresse</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>code_postal</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>conducteur_nom</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>conducteur_naissance</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>conducteur_permis</t>
         </is>
       </c>
     </row>
@@ -494,29 +587,84 @@
           <t>Hilux</t>
         </is>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>VP</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
         <v>2023</v>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Diesel</t>
         </is>
       </c>
-      <c r="G2" t="n">
+      <c r="H2" t="n">
         <v>7</v>
       </c>
-      <c r="H2" t="n">
+      <c r="I2" t="n">
         <v>5</v>
       </c>
-      <c r="I2" t="n">
+      <c r="J2" t="n">
         <v>35000000</v>
       </c>
-      <c r="J2" t="n">
+      <c r="K2" t="n">
         <v>32000000</v>
       </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>VP</t>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Pick-up</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>SARL Transport Log</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>+237612345678</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>contact@transportlog.cm</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Douala</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Rue 12, Bonanjo</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>BP 1234</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>Jean Mbarga</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>1985-06-15</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>2010-01-10</t>
         </is>
       </c>
     </row>
@@ -541,29 +689,84 @@
           <t>Kangoo</t>
         </is>
       </c>
-      <c r="E3" t="n">
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>VU</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
         <v>2022</v>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>Diesel</t>
         </is>
       </c>
-      <c r="G3" t="n">
+      <c r="H3" t="n">
         <v>5</v>
       </c>
-      <c r="H3" t="n">
+      <c r="I3" t="n">
         <v>3</v>
       </c>
-      <c r="I3" t="n">
+      <c r="J3" t="n">
         <v>18000000</v>
       </c>
-      <c r="J3" t="n">
+      <c r="K3" t="n">
         <v>15000000</v>
       </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>VU</t>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Utilitaire</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>SARL Express</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>+237623456789</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>info@express.cm</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>Yaoundé</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>Bastos</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>BP 5678</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>Paul Nganou</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>1990-03-22</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>2012-05-20</t>
         </is>
       </c>
     </row>
@@ -588,29 +791,814 @@
           <t>Outlander</t>
         </is>
       </c>
-      <c r="E4" t="n">
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>VP</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
         <v>2024</v>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>Essence</t>
         </is>
       </c>
-      <c r="G4" t="n">
+      <c r="H4" t="n">
         <v>6</v>
       </c>
-      <c r="H4" t="n">
+      <c r="I4" t="n">
         <v>7</v>
       </c>
-      <c r="I4" t="n">
+      <c r="J4" t="n">
         <v>28000000</v>
       </c>
-      <c r="J4" t="n">
+      <c r="K4" t="n">
         <v>26000000</v>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>SUV</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>ETS Voyages</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>+237634567890</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>contact@voyages.cm</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Douala</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Akwa</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>BP 9012</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>Marie Ngo</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>1988-11-10</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>2011-09-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>LT-004-DE</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>VF4QRSTU12345678</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Peugeot</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>VU</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>2023</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Diesel</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>4</v>
+      </c>
+      <c r="I5" t="n">
+        <v>5</v>
+      </c>
+      <c r="J5" t="n">
+        <v>22000000</v>
+      </c>
+      <c r="K5" t="n">
+        <v>20000000</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Utilitaire</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Logistique Plus</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>+237645678901</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>info@logplus.cm</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Garoua</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>Quartier Administratif</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>BP 3456</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>Jacques Tchoffo</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>1982-08-05</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>2008-03-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>LT-005-EF</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>VF5VWXYZ98765432</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Mercedes</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Sprinter</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>2022</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Diesel</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>8</v>
+      </c>
+      <c r="I6" t="n">
+        <v>9</v>
+      </c>
+      <c r="J6" t="n">
+        <v>45000000</v>
+      </c>
+      <c r="K6" t="n">
+        <v>42000000</v>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Minibus</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Transport SARL</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>+237656789012</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>contact@transport.cm</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Douala</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>Bonabéri</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>BP 7890</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>Emmanuel Njoya</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>1979-12-18</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>2005-06-25</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Colonne</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Exemple</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Statut</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>immatriculation</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>🔴 OBLIGATOIRE - Plaque d'immatriculation du véhicule</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>LT-001-AB</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>🔴 Requis</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>chassis</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Numéro de châssis (17 caractères recommandé)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>VF1ABCDEF12345678</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Optionnel</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>marque</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>🔴 OBLIGATOIRE - Marque du véhicule</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Toyota</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>🔴 Requis</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>modele</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>🔴 OBLIGATOIRE - Modèle du véhicule</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Hilux</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>🔴 Requis</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>categorie</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Catégorie: VP (Véhicule Particulier), VU (Véhicule Utilitaire), PL (Poids Lourd)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
         <is>
           <t>VP</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Recommandé</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>annee</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Année de mise en circulation</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Optionnel</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>energie</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Type d'énergie: Essence, Diesel, Electrique, Hybride</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Diesel</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Recommandé</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>puissance</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Puissance fiscale en CV</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Recommandé</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>places</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Nombre de places assises</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Optionnel</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>valeur_neuf</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Valeur à neuf du véhicule (FCFA)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>35000000</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Recommandé</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>valeur_venale</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Valeur vénale actuelle (FCFA)</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>32000000</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Recommandé</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>type_vehicule</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Type de véhicule: Pick-up, Utilitaire, SUV, Minibus, etc.</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Pick-up</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Optionnel</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>zone_tarifaire</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Zone tarifaire: A, B, C</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Optionnel</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>proprietaire</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Nom du propriétaire (optionnel)</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>SARL Transport Log</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Optionnel</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>telephone</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Téléphone du propriétaire (optionnel)</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>+237612345678</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Optionnel</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Email du propriétaire (optionnel)</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>contact@transportlog.cm</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Optionnel</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>ville</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Ville de résidence</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Douala</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Optionnel</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>adresse</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Adresse complète</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Rue 12, Bonanjo</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Optionnel</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>code_postal</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Code postal / BP</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>BP 1234</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Optionnel</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>conducteur_nom</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Nom du conducteur principal</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Jean Mbarga</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Optionnel</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>conducteur_naissance</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Date de naissance du conducteur (YYYY-MM-DD)</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>1985-06-15</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Optionnel</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>conducteur_permis</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Date d'obtention du permis (YYYY-MM-DD)</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>2010-01-10</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Optionnel</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Logiciel LOMETA complet avec gestion de flotte, et API ASAC. logiciel modulaire permettant d'installer des extentions de vos propres modules. systeme de backup installable. Service de mise à jour complêt pour le suivit des versions installées chez les clients en devenir.
</commit_message>
<xml_diff>
--- a/modele_flotte_import.xlsx
+++ b/modele_flotte_import.xlsx
@@ -427,184 +427,198 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V6"/>
+  <dimension ref="A1:Y6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="17" customWidth="1" min="1" max="1"/>
-    <col width="19" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="7" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="8" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="27" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="6" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
     <col width="15" customWidth="1" min="11" max="11"/>
-    <col width="15" customWidth="1" min="12" max="12"/>
-    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="36" customWidth="1" min="12" max="12"/>
+    <col width="8" customWidth="1" min="13" max="13"/>
     <col width="20" customWidth="1" min="14" max="14"/>
-    <col width="15" customWidth="1" min="15" max="15"/>
-    <col width="25" customWidth="1" min="16" max="16"/>
-    <col width="9" customWidth="1" min="17" max="17"/>
-    <col width="24" customWidth="1" min="18" max="18"/>
-    <col width="13" customWidth="1" min="19" max="19"/>
-    <col width="17" customWidth="1" min="20" max="20"/>
-    <col width="22" customWidth="1" min="21" max="21"/>
-    <col width="19" customWidth="1" min="22" max="22"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="10" customWidth="1" min="17" max="17"/>
+    <col width="16" customWidth="1" min="18" max="18"/>
+    <col width="28" customWidth="1" min="19" max="19"/>
+    <col width="25" customWidth="1" min="20" max="20"/>
+    <col width="18" customWidth="1" min="21" max="21"/>
+    <col width="13" customWidth="1" min="22" max="22"/>
+    <col width="12" customWidth="1" min="23" max="23"/>
+    <col width="13" customWidth="1" min="24" max="24"/>
+    <col width="28" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>immatriculation</t>
+          <t>Rang</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>chassis</t>
+          <t>Immatriculation</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>marque</t>
+          <t>Marque et Type</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>modele</t>
+          <t>Genre</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>categorie</t>
+          <t>Puissance en CV</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>annee</t>
+          <t>Usage</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>energie</t>
+          <t>Nombre de Places</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>puissance</t>
+          <t>Nombre de jours assurés</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>places</t>
+          <t>PMEC</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>valeur_neuf</t>
+          <t>Valeur Neuve</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>valeur_venale</t>
+          <t>Valeur Venale</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>type_vehicule</t>
+          <t>Capital Assistance à la réparation</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>zone_tarifaire</t>
+          <t>RC/RTI</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>proprietaire</t>
+          <t>Défense et Recours</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>telephone</t>
+          <t>Vol/Vol partie</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>email</t>
+          <t>Vol Braquage</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>ville</t>
+          <t>Incendie</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>adresse</t>
+          <t>Bris de Glaces</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
-          <t>code_postal</t>
+          <t>Assistance à la réparation</t>
         </is>
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>conducteur_nom</t>
+          <t>Dommages Tous Accidents</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>conducteur_naissance</t>
+          <t>IPT + Conducteur</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>conducteur_permis</t>
+          <t>Prime brute</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>Réductions</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>Prime nette</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>Droit de Timbre Automobile</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
         <is>
           <t>LT-001-AB</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>VF1ABCDEF12345678</t>
-        </is>
-      </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Toyota</t>
+          <t>Toyota Hilux</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Hilux</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
           <t>VP</t>
         </is>
       </c>
-      <c r="F2" t="n">
-        <v>2023</v>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Diesel</t>
-        </is>
+      <c r="E2" t="n">
+        <v>7</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Transport de personnes</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>5</v>
       </c>
       <c r="H2" t="n">
-        <v>7</v>
+        <v>365</v>
       </c>
       <c r="I2" t="n">
-        <v>5</v>
+        <v>2000</v>
       </c>
       <c r="J2" t="n">
         <v>35000000</v>
@@ -612,101 +626,84 @@
       <c r="K2" t="n">
         <v>32000000</v>
       </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>Pick-up</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>SARL Transport Log</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>+237612345678</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>contact@transportlog.cm</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>Douala</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>Rue 12, Bonanjo</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>BP 1234</t>
-        </is>
-      </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>Jean Mbarga</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>1985-06-15</t>
-        </is>
-      </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>2010-01-10</t>
-        </is>
+      <c r="L2" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>5000</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
         <is>
           <t>LT-002-BC</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>VF2GHIJKL98765432</t>
-        </is>
-      </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Renault</t>
+          <t>Renault Kangoo</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Kangoo</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
           <t>VU</t>
         </is>
       </c>
-      <c r="F3" t="n">
-        <v>2022</v>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Diesel</t>
-        </is>
+      <c r="E3" t="n">
+        <v>5</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Transport de marchandises</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>3</v>
       </c>
       <c r="H3" t="n">
-        <v>5</v>
+        <v>365</v>
       </c>
       <c r="I3" t="n">
-        <v>3</v>
+        <v>1200</v>
       </c>
       <c r="J3" t="n">
         <v>18000000</v>
@@ -714,101 +711,84 @@
       <c r="K3" t="n">
         <v>15000000</v>
       </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>Utilitaire</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>SARL Express</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>+237623456789</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>info@express.cm</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>Yaoundé</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>Bastos</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>BP 5678</t>
-        </is>
-      </c>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>Paul Nganou</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>1990-03-22</t>
-        </is>
-      </c>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t>2012-05-20</t>
-        </is>
+      <c r="L3" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R3" t="n">
+        <v>0</v>
+      </c>
+      <c r="S3" t="n">
+        <v>0</v>
+      </c>
+      <c r="T3" t="n">
+        <v>0</v>
+      </c>
+      <c r="U3" t="n">
+        <v>0</v>
+      </c>
+      <c r="V3" t="n">
+        <v>0</v>
+      </c>
+      <c r="W3" t="n">
+        <v>0</v>
+      </c>
+      <c r="X3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>5000</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
         <is>
           <t>LT-003-CD</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>VF3MNOPQR45678901</t>
-        </is>
-      </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Mitsubishi</t>
+          <t>Mitsubishi Outlander</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Outlander</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
           <t>VP</t>
         </is>
       </c>
-      <c r="F4" t="n">
-        <v>2024</v>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Essence</t>
-        </is>
+      <c r="E4" t="n">
+        <v>6</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Transport de personnes</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>7</v>
       </c>
       <c r="H4" t="n">
-        <v>6</v>
+        <v>365</v>
       </c>
       <c r="I4" t="n">
-        <v>7</v>
+        <v>1800</v>
       </c>
       <c r="J4" t="n">
         <v>28000000</v>
@@ -816,101 +796,84 @@
       <c r="K4" t="n">
         <v>26000000</v>
       </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>SUV</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>ETS Voyages</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>+237634567890</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>contact@voyages.cm</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>Douala</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>Akwa</t>
-        </is>
-      </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>BP 9012</t>
-        </is>
-      </c>
-      <c r="T4" t="inlineStr">
-        <is>
-          <t>Marie Ngo</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>1988-11-10</t>
-        </is>
-      </c>
-      <c r="V4" t="inlineStr">
-        <is>
-          <t>2011-09-15</t>
-        </is>
+      <c r="L4" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V4" t="n">
+        <v>0</v>
+      </c>
+      <c r="W4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>5000</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
         <is>
           <t>LT-004-DE</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>VF4QRSTU12345678</t>
-        </is>
-      </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Peugeot</t>
+          <t>Peugeot Partner</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Partner</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
           <t>VU</t>
         </is>
       </c>
-      <c r="F5" t="n">
-        <v>2023</v>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Diesel</t>
-        </is>
+      <c r="E5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Transport de marchandises</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>5</v>
       </c>
       <c r="H5" t="n">
-        <v>4</v>
+        <v>365</v>
       </c>
       <c r="I5" t="n">
-        <v>5</v>
+        <v>1500</v>
       </c>
       <c r="J5" t="n">
         <v>22000000</v>
@@ -918,101 +881,84 @@
       <c r="K5" t="n">
         <v>20000000</v>
       </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>Utilitaire</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>Logistique Plus</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>+237645678901</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>info@logplus.cm</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>Garoua</t>
-        </is>
-      </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>Quartier Administratif</t>
-        </is>
-      </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>BP 3456</t>
-        </is>
-      </c>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>Jacques Tchoffo</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>1982-08-05</t>
-        </is>
-      </c>
-      <c r="V5" t="inlineStr">
-        <is>
-          <t>2008-03-12</t>
-        </is>
+      <c r="L5" t="n">
+        <v>3500000</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S5" t="n">
+        <v>0</v>
+      </c>
+      <c r="T5" t="n">
+        <v>0</v>
+      </c>
+      <c r="U5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V5" t="n">
+        <v>0</v>
+      </c>
+      <c r="W5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>5000</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
         <is>
           <t>LT-005-EF</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>VF5VWXYZ98765432</t>
-        </is>
-      </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Mercedes</t>
+          <t>Mercedes Sprinter</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Sprinter</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
           <t>PL</t>
         </is>
       </c>
-      <c r="F6" t="n">
-        <v>2022</v>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Diesel</t>
-        </is>
+      <c r="E6" t="n">
+        <v>8</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Transport de personnes</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>9</v>
       </c>
       <c r="H6" t="n">
-        <v>8</v>
+        <v>365</v>
       </c>
       <c r="I6" t="n">
-        <v>9</v>
+        <v>3500</v>
       </c>
       <c r="J6" t="n">
         <v>45000000</v>
@@ -1020,60 +966,47 @@
       <c r="K6" t="n">
         <v>42000000</v>
       </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>Minibus</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>Transport SARL</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>+237656789012</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>contact@transport.cm</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>Douala</t>
-        </is>
-      </c>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>Bonabéri</t>
-        </is>
-      </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>BP 7890</t>
-        </is>
-      </c>
-      <c r="T6" t="inlineStr">
-        <is>
-          <t>Emmanuel Njoya</t>
-        </is>
-      </c>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>1979-12-18</t>
-        </is>
-      </c>
-      <c r="V6" t="inlineStr">
-        <is>
-          <t>2005-06-25</t>
-        </is>
+      <c r="L6" t="n">
+        <v>6000000</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V6" t="n">
+        <v>0</v>
+      </c>
+      <c r="W6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>5000</v>
       </c>
     </row>
   </sheetData>
@@ -1087,13 +1020,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="50" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1109,11 +1041,6 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Exemple</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
           <t>Statut</t>
         </is>
       </c>
@@ -1121,64 +1048,49 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>immatriculation</t>
+          <t>Rang</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>🔴 OBLIGATOIRE - Plaque d'immatriculation du véhicule</t>
+          <t>Numéro de rang (optionnel)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>LT-001-AB</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>🔴 Requis</t>
+          <t>Optionnel</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>chassis</t>
+          <t>Immatriculation</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Numéro de châssis (17 caractères recommandé)</t>
+          <t>🔴 OBLIGATOIRE - Plaque d'immatriculation</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>VF1ABCDEF12345678</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Optionnel</t>
+          <t>🔴 Requis</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>marque</t>
+          <t>Marque et Type</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>🔴 OBLIGATOIRE - Marque du véhicule</t>
+          <t>🔴 OBLIGATOIRE - Marque et modèle du véhicule</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
-        <is>
-          <t>Toyota</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
         <is>
           <t>🔴 Requis</t>
         </is>
@@ -1187,42 +1099,32 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>modele</t>
+          <t>Genre</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>🔴 OBLIGATOIRE - Modèle du véhicule</t>
+          <t>Genre du véhicule (VP, VU, PL, etc.)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Hilux</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>🔴 Requis</t>
+          <t>Recommandé</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>categorie</t>
+          <t>Puissance en CV</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Catégorie: VP (Véhicule Particulier), VU (Véhicule Utilitaire), PL (Poids Lourd)</t>
+          <t>Puissance fiscale en CV</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
-        <is>
-          <t>VP</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
         <is>
           <t>Recommandé</t>
         </is>
@@ -1231,20 +1133,15 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>annee</t>
+          <t>Usage</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Année de mise en circulation</t>
+          <t>Usage du véhicule</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
-        <is>
-          <t>2023</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
         <is>
           <t>Optionnel</t>
         </is>
@@ -1253,20 +1150,15 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>energie</t>
+          <t>Nombre de Places</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Type d'énergie: Essence, Diesel, Electrique, Hybride</t>
+          <t>Nombre de places assises</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
-        <is>
-          <t>Diesel</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
         <is>
           <t>Recommandé</t>
         </is>
@@ -1275,42 +1167,32 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>puissance</t>
+          <t>Nombre de jours assurés</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Puissance fiscale en CV</t>
+          <t>Nombre de jours d'assurance (365 par défaut)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Recommandé</t>
+          <t>Optionnel</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>places</t>
+          <t>PMEC</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Nombre de places assises</t>
+          <t>PMEC (Poids Maximum Autorisé)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
         <is>
           <t>Optionnel</t>
         </is>
@@ -1319,7 +1201,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>valeur_neuf</t>
+          <t>Valeur Neuve</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1328,11 +1210,6 @@
         </is>
       </c>
       <c r="C11" t="inlineStr">
-        <is>
-          <t>35000000</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
         <is>
           <t>Recommandé</t>
         </is>
@@ -1341,7 +1218,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>valeur_venale</t>
+          <t>Valeur Venale</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1350,11 +1227,6 @@
         </is>
       </c>
       <c r="C12" t="inlineStr">
-        <is>
-          <t>32000000</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
         <is>
           <t>Recommandé</t>
         </is>
@@ -1363,20 +1235,15 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>type_vehicule</t>
+          <t>Capital Assistance à la réparation</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Type de véhicule: Pick-up, Utilitaire, SUV, Minibus, etc.</t>
+          <t>Capital pour l'assistance à la réparation</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
-        <is>
-          <t>Pick-up</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
         <is>
           <t>Optionnel</t>
         </is>
@@ -1385,20 +1252,15 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>zone_tarifaire</t>
+          <t>RC/RTI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Zone tarifaire: A, B, C</t>
+          <t>RC/RTI - Laisser 0 pour calcul automatique</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
         <is>
           <t>Optionnel</t>
         </is>
@@ -1407,20 +1269,15 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>proprietaire</t>
+          <t>Défense et Recours</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Nom du propriétaire (optionnel)</t>
+          <t>Défense et Recours - Laisser 0 pour calcul automatique</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
-        <is>
-          <t>SARL Transport Log</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
         <is>
           <t>Optionnel</t>
         </is>
@@ -1429,20 +1286,15 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>telephone</t>
+          <t>Vol/Vol partie</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Téléphone du propriétaire (optionnel)</t>
+          <t>Vol/Vol partie - Laisser 0 pour calcul automatique</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
-        <is>
-          <t>+237612345678</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
         <is>
           <t>Optionnel</t>
         </is>
@@ -1451,20 +1303,15 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>email</t>
+          <t>Vol Braquage</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Email du propriétaire (optionnel)</t>
+          <t>Vol Braquage - Laisser 0 pour calcul automatique</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
-        <is>
-          <t>contact@transportlog.cm</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
         <is>
           <t>Optionnel</t>
         </is>
@@ -1473,20 +1320,15 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ville</t>
+          <t>Incendie</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Ville de résidence</t>
+          <t>Incendie - Laisser 0 pour calcul automatique</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
-        <is>
-          <t>Douala</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
         <is>
           <t>Optionnel</t>
         </is>
@@ -1495,20 +1337,15 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>adresse</t>
+          <t>Bris de Glaces</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Adresse complète</t>
+          <t>Bris de Glaces - Laisser 0 pour calcul automatique</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
-        <is>
-          <t>Rue 12, Bonanjo</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
         <is>
           <t>Optionnel</t>
         </is>
@@ -1517,20 +1354,15 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>code_postal</t>
+          <t>Assistance à la réparation</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Code postal / BP</t>
+          <t>Assistance à la réparation - Laisser 0 pour calcul automatique</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
-        <is>
-          <t>BP 1234</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
         <is>
           <t>Optionnel</t>
         </is>
@@ -1539,20 +1371,15 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>conducteur_nom</t>
+          <t>Dommages Tous Accidents</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Nom du conducteur principal</t>
+          <t>Dommages Tous Accidents - Laisser 0 pour calcul automatique</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
-        <is>
-          <t>Jean Mbarga</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
         <is>
           <t>Optionnel</t>
         </is>
@@ -1561,20 +1388,15 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>conducteur_naissance</t>
+          <t>IPT + Conducteur</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Date de naissance du conducteur (YYYY-MM-DD)</t>
+          <t>IPT + Conducteur - Laisser 0 pour calcul automatique</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
-        <is>
-          <t>1985-06-15</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
         <is>
           <t>Optionnel</t>
         </is>
@@ -1583,20 +1405,66 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>conducteur_permis</t>
+          <t>Prime brute</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Date d'obtention du permis (YYYY-MM-DD)</t>
+          <t>Prime brute - Laisser 0 pour calcul automatique</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2010-01-10</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
+          <t>Optionnel</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Réductions</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Réductions - Appliquer manuellement si besoin</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Optionnel</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Prime nette</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Prime nette - Laisser 0 pour calcul automatique</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Optionnel</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Droit de Timbre Automobile</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Droit de Timbre Automobile (5000 FCFA par défaut)</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
         <is>
           <t>Optionnel</t>
         </is>

</xml_diff>